<commit_message>
Calculation updated with crime effects, Dash layout updated with navi bar
</commit_message>
<xml_diff>
--- a/Data/Spreadsheets/subcomponent_scenarios_plus_descriptionsv2.xlsx
+++ b/Data/Spreadsheets/subcomponent_scenarios_plus_descriptionsv2.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/Spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/Spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACD4EE0-BD56-204A-9E9D-5AF786977C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C17C79A8-3CEB-334C-9DDF-236C738AF772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="1540" windowWidth="29260" windowHeight="16100" xr2:uid="{E3CEDC4D-39E8-6049-89E8-D0BEF71875A0}"/>
+    <workbookView xWindow="140" yWindow="1540" windowWidth="29260" windowHeight="16100" activeTab="1" xr2:uid="{E3CEDC4D-39E8-6049-89E8-D0BEF71875A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="128">
   <si>
     <t>Det Value</t>
   </si>
@@ -363,13 +364,457 @@
   </si>
   <si>
     <t>Choose if you think detention harms communities but may reduce crime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  # Remove these lines from get_scenario_description():</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  'reduced_crime': 'Models a scenario where crime rates decrease...',</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  'increased_crime': 'Models a scenario where crime rates increase...',</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  'diversion_program': 'Simulates the impact of implementing pre-trial diversion programs...',</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  'bail_reform': 'Models the effects of bail reform policies...',</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  'capacity_expansion': 'Analyzes the impact of expanding facility capacity...'</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">def </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF56A8F5"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>_get_scenario_description</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>(scenario):</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF5F826B"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>"""Return the description for a given scenario."""</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>descriptions = {</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'baseline'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Represents current operations at Cook County Jail with standard parameters. This scenario serves as the reference point for comparison.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'most conservative'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Uses conservative estimates for all parameters, minimizing potential benefits and maximizing costs. Provides a lower-bound estimate of MVPF.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'least conservative'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Uses optimistic estimates that maximize potential benefits and minimize costs. Provides an upper-bound estimate of MVPF.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'reduced_crime'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Models a scenario where crime rates decrease, resulting in lower detention demand and associated costs.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'increased_crime'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Models a scenario where crime rates increase, resulting in higher detention demand and associated costs.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'diversion_program'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Simulates the impact of implementing pre-trial diversion programs that reduce jail population through alternative interventions.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'bail_reform'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Models the effects of bail reform policies that reduce pretrial detention for low-risk individuals.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">        </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'capacity_expansion'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'Analyzes the impact of expanding facility capacity to accommodate more detainees.'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFCF8E6D"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">return </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve">descriptions.get(scenario, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FF6AAB73"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>'No description available for this scenario.'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.8000000000000007"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -443,6 +888,37 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFCF8E6D"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF56A8F5"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF5F826B"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF6AAB73"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -464,7 +940,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -497,6 +973,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -832,7 +1312,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE80E8B-CEB2-B84F-9C91-FD8EDADFF9F9}">
   <dimension ref="A1:M43"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="24" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="24"/>
   <cols>
     <col min="1" max="1" width="76.5" customWidth="1"/>
     <col min="2" max="2" width="31" customWidth="1"/>
@@ -845,7 +1325,7 @@
     <col min="11" max="11" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="25">
       <c r="A1" s="6" t="s">
         <v>20</v>
       </c>
@@ -865,10 +1345,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13">
       <c r="A2" s="6"/>
     </row>
-    <row r="3" spans="1:13" s="2" customFormat="1" ht="300" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" s="2" customFormat="1" ht="300">
       <c r="A3" s="2" t="s">
         <v>45</v>
       </c>
@@ -904,7 +1384,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="200" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="200">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -942,7 +1422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="275" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="275">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -977,7 +1457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="325" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="325">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -1015,7 +1495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="200" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="200">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -1054,7 +1534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="200" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="200">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -1092,7 +1572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="175" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="175">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1130,7 +1610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="175" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="175">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -1165,7 +1645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="300" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="300">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1203,7 +1683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="275" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="275">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1238,7 +1718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1246,7 +1726,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="50" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ht="50">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -1257,12 +1737,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="25">
       <c r="D16" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6">
       <c r="A18" s="7" t="s">
         <v>20</v>
       </c>
@@ -1276,7 +1756,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="225" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="225">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -1284,7 +1764,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="125">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -1295,7 +1775,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="200" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="200">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1306,7 +1786,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="175" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="175">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -1320,7 +1800,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:6" s="5" customFormat="1" ht="125" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" s="5" customFormat="1" ht="125">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -1336,7 +1816,7 @@
       <c r="E23" s="14"/>
       <c r="F23" s="14"/>
     </row>
-    <row r="24" spans="1:6" ht="150" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="150">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -1347,7 +1827,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="150" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="150">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -1358,7 +1838,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="125">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -1369,7 +1849,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="125">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -1383,7 +1863,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="150" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="150">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -1394,7 +1874,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:6" s="3" customFormat="1" ht="25" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" s="3" customFormat="1" ht="25">
       <c r="A32" s="8" t="s">
         <v>20</v>
       </c>
@@ -1410,7 +1890,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="275" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" ht="275">
       <c r="A33" s="9" t="s">
         <v>46</v>
       </c>
@@ -1421,7 +1901,7 @@
       <c r="E33" s="11"/>
       <c r="F33" s="11"/>
     </row>
-    <row r="34" spans="1:6" ht="100" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="100">
       <c r="A34" s="9" t="s">
         <v>33</v>
       </c>
@@ -1441,7 +1921,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="150" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" ht="100">
       <c r="A35" s="9" t="s">
         <v>34</v>
       </c>
@@ -1459,7 +1939,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" ht="75">
       <c r="A36" s="9" t="s">
         <v>35</v>
       </c>
@@ -1479,7 +1959,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="100" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" ht="100">
       <c r="A37" s="9" t="s">
         <v>24</v>
       </c>
@@ -1499,7 +1979,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" ht="75">
       <c r="A38" s="9" t="s">
         <v>25</v>
       </c>
@@ -1519,7 +1999,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="100" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="75">
       <c r="A39" s="9" t="s">
         <v>26</v>
       </c>
@@ -1539,7 +2019,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="75" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" ht="75">
       <c r="A40" s="9" t="s">
         <v>27</v>
       </c>
@@ -1557,7 +2037,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" ht="100">
       <c r="A41" s="9" t="s">
         <v>28</v>
       </c>
@@ -1577,7 +2057,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="125" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" ht="75">
       <c r="A42" s="9" t="s">
         <v>29</v>
       </c>
@@ -1595,7 +2075,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6">
       <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="11"/>
@@ -1606,4 +2086,109 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBEF1827-83DA-914B-9108-04A20EBE7F7F}">
+  <dimension ref="A2:A23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetData>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="17" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="17" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="17" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="17" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="19" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="17" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>